<commit_message>
added compliance map for Soc2 type 2
</commit_message>
<xml_diff>
--- a/Audit_Code/public/SOC2_Type2.xlsx
+++ b/Audit_Code/public/SOC2_Type2.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Compliance\Audit_Code\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muhammad.abdullah\Documents\Compliance\Audit_Code\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4635"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15348" windowHeight="4632"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$D$1:$F$94</definedName>
   </definedNames>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3">
     <font>
       <sz val="11"/>
@@ -1134,18 +1134,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F94"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="9.125" style="9"/>
-    <col min="2" max="2" width="29.625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="8.875" style="9" customWidth="1"/>
-    <col min="4" max="4" width="37.125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="7.875" style="9" customWidth="1"/>
-    <col min="6" max="6" width="107.125" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.125" style="2"/>
+    <col min="1" max="1" width="9.09765625" style="9"/>
+    <col min="2" max="2" width="29.59765625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="8.8984375" style="9" customWidth="1"/>
+    <col min="4" max="4" width="37.09765625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="7.8984375" style="9" customWidth="1"/>
+    <col min="6" max="6" width="107.09765625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.09765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" ht="15">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="7"/>
       <c r="B1" s="3" t="s">
         <v>107</v>
@@ -1199,7 +1199,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="28.5">
+    <row r="4" spans="1:6" ht="27.6">
       <c r="A4" s="8">
         <v>2</v>
       </c>
@@ -1279,7 +1279,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="28.5">
+    <row r="8" spans="1:6" ht="27.6">
       <c r="A8" s="8">
         <v>2</v>
       </c>
@@ -1319,7 +1319,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="42.75">
+    <row r="10" spans="1:6" ht="41.4">
       <c r="A10" s="8">
         <v>2</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="28.5">
+    <row r="11" spans="1:6" ht="27.6">
       <c r="A11" s="8">
         <v>2</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="42.75">
+    <row r="12" spans="1:6" ht="41.4">
       <c r="A12" s="8">
         <v>3</v>
       </c>
@@ -1379,7 +1379,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="28.5">
+    <row r="13" spans="1:6" ht="27.6">
       <c r="A13" s="8">
         <v>3</v>
       </c>
@@ -1407,14 +1407,12 @@
         <v>40</v>
       </c>
       <c r="C14" s="8">
-        <f t="shared" ref="C14:C35" si="0">C13+0.1</f>
-        <v>3.3000000000000003</v>
+        <v>3.3</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>121</v>
       </c>
       <c r="E14" s="8">
-        <f t="shared" ref="E4:E67" si="1">E13+1</f>
         <v>13</v>
       </c>
       <c r="F14" s="5" t="s">
@@ -1429,21 +1427,19 @@
         <v>40</v>
       </c>
       <c r="C15" s="8">
-        <f t="shared" si="0"/>
-        <v>3.4000000000000004</v>
+        <v>3.4</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>122</v>
       </c>
       <c r="E15" s="8">
-        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="28.5">
+    <row r="16" spans="1:6" ht="27.6">
       <c r="A16" s="8">
         <v>3</v>
       </c>
@@ -1451,21 +1447,19 @@
         <v>40</v>
       </c>
       <c r="C16" s="8">
-        <f t="shared" si="0"/>
-        <v>3.5000000000000004</v>
+        <v>3.5</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>123</v>
       </c>
       <c r="E16" s="8">
-        <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="42.75">
+    <row r="17" spans="1:6" ht="41.4">
       <c r="A17" s="8">
         <v>3</v>
       </c>
@@ -1473,14 +1467,12 @@
         <v>40</v>
       </c>
       <c r="C17" s="8">
-        <f t="shared" si="0"/>
-        <v>3.6000000000000005</v>
+        <v>3.6</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>124</v>
       </c>
       <c r="E17" s="8">
-        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="F17" s="4" t="s">
@@ -1501,14 +1493,13 @@
         <v>140</v>
       </c>
       <c r="E18" s="8">
-        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="28.5">
+    <row r="19" spans="1:6" ht="27.6">
       <c r="A19" s="8">
         <v>4</v>
       </c>
@@ -1516,21 +1507,19 @@
         <v>18</v>
       </c>
       <c r="C19" s="8">
-        <f t="shared" si="0"/>
-        <v>4.1999999999999993</v>
+        <v>4.2</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>141</v>
       </c>
       <c r="E19" s="8">
-        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="28.5">
+    <row r="20" spans="1:6" ht="27.6">
       <c r="A20" s="8">
         <v>4</v>
       </c>
@@ -1538,21 +1527,19 @@
         <v>18</v>
       </c>
       <c r="C20" s="8">
-        <f t="shared" si="0"/>
-        <v>4.2999999999999989</v>
+        <v>4.3</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>142</v>
       </c>
       <c r="E20" s="8">
-        <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="42.75">
+    <row r="21" spans="1:6" ht="41.4">
       <c r="A21" s="8">
         <v>4</v>
       </c>
@@ -1560,21 +1547,19 @@
         <v>18</v>
       </c>
       <c r="C21" s="8">
-        <f t="shared" si="0"/>
-        <v>4.3999999999999986</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>143</v>
       </c>
       <c r="E21" s="8">
-        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="28.5">
+    <row r="22" spans="1:6" ht="27.6">
       <c r="A22" s="8">
         <v>4</v>
       </c>
@@ -1582,21 +1567,19 @@
         <v>18</v>
       </c>
       <c r="C22" s="8">
-        <f t="shared" si="0"/>
-        <v>4.4999999999999982</v>
+        <v>4.5</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>144</v>
       </c>
       <c r="E22" s="8">
-        <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="28.5">
+    <row r="23" spans="1:6" ht="27.6">
       <c r="A23" s="8">
         <v>4</v>
       </c>
@@ -1604,21 +1587,19 @@
         <v>18</v>
       </c>
       <c r="C23" s="8">
-        <f t="shared" si="0"/>
-        <v>4.5999999999999979</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>146</v>
       </c>
       <c r="E23" s="8">
-        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="42.75">
+    <row r="24" spans="1:6" ht="41.4">
       <c r="A24" s="8">
         <v>4</v>
       </c>
@@ -1626,21 +1607,19 @@
         <v>18</v>
       </c>
       <c r="C24" s="8">
-        <f t="shared" si="0"/>
-        <v>4.6999999999999975</v>
+        <v>4.7</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>148</v>
       </c>
       <c r="E24" s="8">
-        <f t="shared" si="1"/>
         <v>23</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="28.5">
+    <row r="25" spans="1:6" ht="27.6">
       <c r="A25" s="8">
         <v>4</v>
       </c>
@@ -1648,21 +1627,19 @@
         <v>18</v>
       </c>
       <c r="C25" s="8">
-        <f t="shared" si="0"/>
-        <v>4.7999999999999972</v>
+        <v>4.8</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>149</v>
       </c>
       <c r="E25" s="8">
-        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="28.5">
+    <row r="26" spans="1:6" ht="27.6">
       <c r="A26" s="8">
         <v>5</v>
       </c>
@@ -1676,14 +1653,13 @@
         <v>150</v>
       </c>
       <c r="E26" s="8">
-        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="28.5">
+    <row r="27" spans="1:6" ht="27.6">
       <c r="A27" s="8">
         <v>5</v>
       </c>
@@ -1691,21 +1667,19 @@
         <v>5</v>
       </c>
       <c r="C27" s="8">
-        <f t="shared" si="0"/>
         <v>5.0999999999999996</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>151</v>
       </c>
       <c r="E27" s="8">
-        <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="42.75">
+    <row r="28" spans="1:6" ht="41.4">
       <c r="A28" s="8">
         <v>5</v>
       </c>
@@ -1713,21 +1687,19 @@
         <v>5</v>
       </c>
       <c r="C28" s="8">
-        <f t="shared" si="0"/>
-        <v>5.1999999999999993</v>
+        <v>5.2</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>152</v>
       </c>
       <c r="E28" s="8">
-        <f t="shared" si="1"/>
         <v>27</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="28.5">
+    <row r="29" spans="1:6" ht="27.6">
       <c r="A29" s="8">
         <v>5</v>
       </c>
@@ -1735,21 +1707,19 @@
         <v>5</v>
       </c>
       <c r="C29" s="8">
-        <f t="shared" si="0"/>
-        <v>5.2999999999999989</v>
+        <v>5.3</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>153</v>
       </c>
       <c r="E29" s="8">
-        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="42.75">
+    <row r="30" spans="1:6" ht="27.6">
       <c r="A30" s="8">
         <v>5</v>
       </c>
@@ -1757,14 +1727,12 @@
         <v>5</v>
       </c>
       <c r="C30" s="8">
-        <f t="shared" si="0"/>
-        <v>5.3999999999999986</v>
+        <v>5.4</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>154</v>
       </c>
       <c r="E30" s="8">
-        <f t="shared" si="1"/>
         <v>29</v>
       </c>
       <c r="F30" s="4" t="s">
@@ -1779,21 +1747,19 @@
         <v>5</v>
       </c>
       <c r="C31" s="8">
-        <f t="shared" si="0"/>
-        <v>5.4999999999999982</v>
+        <v>5.5</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>155</v>
       </c>
       <c r="E31" s="8">
-        <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="28.5">
+    <row r="32" spans="1:6" ht="27.6">
       <c r="A32" s="8">
         <v>5</v>
       </c>
@@ -1801,14 +1767,12 @@
         <v>5</v>
       </c>
       <c r="C32" s="8">
-        <f t="shared" si="0"/>
-        <v>5.5999999999999979</v>
+        <v>5.6</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>156</v>
       </c>
       <c r="E32" s="8">
-        <f t="shared" si="1"/>
         <v>31</v>
       </c>
       <c r="F32" s="4" t="s">
@@ -1823,21 +1787,19 @@
         <v>5</v>
       </c>
       <c r="C33" s="8">
-        <f t="shared" si="0"/>
-        <v>5.6999999999999975</v>
+        <v>5.7</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>157</v>
       </c>
       <c r="E33" s="8">
-        <f t="shared" si="1"/>
         <v>32</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="28.5">
+    <row r="34" spans="1:6" ht="27.6">
       <c r="A34" s="8">
         <v>5</v>
       </c>
@@ -1845,14 +1807,12 @@
         <v>5</v>
       </c>
       <c r="C34" s="8">
-        <f t="shared" si="0"/>
-        <v>5.7999999999999972</v>
+        <v>5.8</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>158</v>
       </c>
       <c r="E34" s="8">
-        <f t="shared" si="1"/>
         <v>33</v>
       </c>
       <c r="F34" s="4" t="s">
@@ -1867,14 +1827,12 @@
         <v>5</v>
       </c>
       <c r="C35" s="8">
-        <f t="shared" si="0"/>
-        <v>5.8999999999999968</v>
+        <v>5.9</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>159</v>
       </c>
       <c r="E35" s="8">
-        <f t="shared" si="1"/>
         <v>34</v>
       </c>
       <c r="F35" s="4" t="s">
@@ -1895,7 +1853,6 @@
         <v>125</v>
       </c>
       <c r="E36" s="8">
-        <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="F36" s="5" t="s">
@@ -1910,21 +1867,19 @@
         <v>92</v>
       </c>
       <c r="C37" s="8">
-        <f t="shared" ref="A36:C53" si="2">C36+1</f>
         <v>7.1</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>126</v>
       </c>
       <c r="E37" s="8">
-        <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="28.5">
+    <row r="38" spans="1:6" ht="27.6">
       <c r="A38" s="8">
         <v>8</v>
       </c>
@@ -1938,14 +1893,13 @@
         <v>160</v>
       </c>
       <c r="E38" s="8">
-        <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="28.5">
+    <row r="39" spans="1:6" ht="27.6">
       <c r="A39" s="8">
         <v>8</v>
       </c>
@@ -1953,21 +1907,19 @@
         <v>90</v>
       </c>
       <c r="C39" s="8">
-        <f t="shared" ref="C39:C45" si="3">C38+0.1</f>
         <v>8.1999999999999993</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>161</v>
       </c>
       <c r="E39" s="8">
-        <f t="shared" si="1"/>
         <v>38</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="28.5">
+    <row r="40" spans="1:6" ht="27.6">
       <c r="A40" s="8">
         <v>8</v>
       </c>
@@ -1975,21 +1927,19 @@
         <v>90</v>
       </c>
       <c r="C40" s="8">
-        <f t="shared" si="3"/>
-        <v>8.2999999999999989</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>162</v>
       </c>
       <c r="E40" s="8">
-        <f t="shared" si="1"/>
         <v>39</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="28.5">
+    <row r="41" spans="1:6" ht="27.6">
       <c r="A41" s="8">
         <v>8</v>
       </c>
@@ -1997,21 +1947,19 @@
         <v>90</v>
       </c>
       <c r="C41" s="8">
-        <f t="shared" si="3"/>
-        <v>8.3999999999999986</v>
+        <v>8.4</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>163</v>
       </c>
       <c r="E41" s="8">
-        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="28.5">
+    <row r="42" spans="1:6" ht="27.6">
       <c r="A42" s="8">
         <v>8</v>
       </c>
@@ -2019,21 +1967,19 @@
         <v>90</v>
       </c>
       <c r="C42" s="8">
-        <f t="shared" si="3"/>
-        <v>8.4999999999999982</v>
+        <v>8.5</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>164</v>
       </c>
       <c r="E42" s="8">
-        <f t="shared" si="1"/>
         <v>41</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="28.5">
+    <row r="43" spans="1:6" ht="27.6">
       <c r="A43" s="8">
         <v>8</v>
       </c>
@@ -2041,21 +1987,19 @@
         <v>90</v>
       </c>
       <c r="C43" s="8">
-        <f t="shared" si="3"/>
-        <v>8.5999999999999979</v>
+        <v>8.6</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>165</v>
       </c>
       <c r="E43" s="8">
-        <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="28.5">
+    <row r="44" spans="1:6" ht="27.6">
       <c r="A44" s="8">
         <v>8</v>
       </c>
@@ -2063,21 +2007,19 @@
         <v>90</v>
       </c>
       <c r="C44" s="8">
-        <f t="shared" si="3"/>
-        <v>8.6999999999999975</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>166</v>
       </c>
       <c r="E44" s="8">
-        <f t="shared" si="1"/>
         <v>43</v>
       </c>
       <c r="F44" s="4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="28.5">
+    <row r="45" spans="1:6" ht="27.6">
       <c r="A45" s="8">
         <v>8</v>
       </c>
@@ -2085,21 +2027,19 @@
         <v>90</v>
       </c>
       <c r="C45" s="8">
-        <f t="shared" si="3"/>
-        <v>8.7999999999999972</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>167</v>
       </c>
       <c r="E45" s="8">
-        <f t="shared" si="1"/>
         <v>44</v>
       </c>
       <c r="F45" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="28.5">
+    <row r="46" spans="1:6" ht="27.6">
       <c r="A46" s="8">
         <v>8</v>
       </c>
@@ -2107,21 +2047,19 @@
         <v>83</v>
       </c>
       <c r="C46" s="8">
-        <f>C45+0.1</f>
-        <v>8.8999999999999968</v>
+        <v>8.9</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>168</v>
       </c>
       <c r="E46" s="8">
-        <f t="shared" si="1"/>
         <v>45</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="28.5">
+    <row r="47" spans="1:6" ht="27.6">
       <c r="A47" s="8">
         <v>8</v>
       </c>
@@ -2135,14 +2073,13 @@
         <v>169</v>
       </c>
       <c r="E47" s="8">
-        <f t="shared" si="1"/>
         <v>46</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="28.5">
+    <row r="48" spans="1:6" ht="27.6">
       <c r="A48" s="8">
         <v>8</v>
       </c>
@@ -2156,14 +2093,13 @@
         <v>170</v>
       </c>
       <c r="E48" s="8">
-        <f t="shared" si="1"/>
         <v>47</v>
       </c>
       <c r="F48" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="28.5">
+    <row r="49" spans="1:6" ht="27.6">
       <c r="A49" s="8">
         <v>9</v>
       </c>
@@ -2177,14 +2113,13 @@
         <v>172</v>
       </c>
       <c r="E49" s="8">
-        <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="F49" s="5" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="28.5">
+    <row r="50" spans="1:6" ht="27.6">
       <c r="A50" s="8">
         <v>10</v>
       </c>
@@ -2192,21 +2127,19 @@
         <v>104</v>
       </c>
       <c r="C50" s="8">
-        <f t="shared" si="2"/>
         <v>10.1</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>173</v>
       </c>
       <c r="E50" s="8">
-        <f t="shared" si="1"/>
         <v>49</v>
       </c>
       <c r="F50" s="4" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="28.5">
+    <row r="51" spans="1:6" ht="27.6">
       <c r="A51" s="8">
         <v>11</v>
       </c>
@@ -2214,21 +2147,19 @@
         <v>105</v>
       </c>
       <c r="C51" s="8">
-        <f t="shared" si="2"/>
         <v>11.1</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>174</v>
       </c>
       <c r="E51" s="8">
-        <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="F51" s="4" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="28.5">
+    <row r="52" spans="1:6" ht="27.6">
       <c r="A52" s="8">
         <v>12</v>
       </c>
@@ -2236,21 +2167,19 @@
         <v>95</v>
       </c>
       <c r="C52" s="8">
-        <f t="shared" si="2"/>
         <v>12.1</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>175</v>
       </c>
       <c r="E52" s="8">
-        <f t="shared" si="1"/>
         <v>51</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="42.75">
+    <row r="53" spans="1:6" ht="41.4">
       <c r="A53" s="8">
         <v>13</v>
       </c>
@@ -2258,21 +2187,19 @@
         <v>106</v>
       </c>
       <c r="C53" s="8">
-        <f t="shared" si="2"/>
         <v>13.1</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>176</v>
       </c>
       <c r="E53" s="8">
-        <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="42.75">
+    <row r="54" spans="1:6" ht="41.4">
       <c r="A54" s="8">
         <v>14</v>
       </c>
@@ -2286,14 +2213,13 @@
         <v>177</v>
       </c>
       <c r="E54" s="8">
-        <f t="shared" si="1"/>
         <v>53</v>
       </c>
       <c r="F54" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="28.5">
+    <row r="55" spans="1:6" ht="27.6">
       <c r="A55" s="8">
         <v>14</v>
       </c>
@@ -2301,21 +2227,19 @@
         <v>28</v>
       </c>
       <c r="C55" s="8">
-        <f t="shared" ref="C55:C62" si="4">C54+0.1</f>
         <v>14.2</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>178</v>
       </c>
       <c r="E55" s="8">
-        <f t="shared" si="1"/>
         <v>54</v>
       </c>
       <c r="F55" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="28.5">
+    <row r="56" spans="1:6" ht="27.6">
       <c r="A56" s="8">
         <v>14</v>
       </c>
@@ -2323,21 +2247,19 @@
         <v>28</v>
       </c>
       <c r="C56" s="8">
-        <f t="shared" si="4"/>
-        <v>14.299999999999999</v>
+        <v>14.3</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>179</v>
       </c>
       <c r="E56" s="8">
-        <f t="shared" si="1"/>
         <v>55</v>
       </c>
       <c r="F56" s="4" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="28.5">
+    <row r="57" spans="1:6" ht="27.6">
       <c r="A57" s="8">
         <v>14</v>
       </c>
@@ -2345,21 +2267,19 @@
         <v>28</v>
       </c>
       <c r="C57" s="8">
-        <f t="shared" si="4"/>
-        <v>14.399999999999999</v>
+        <v>14.4</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>180</v>
       </c>
       <c r="E57" s="8">
-        <f t="shared" si="1"/>
         <v>56</v>
       </c>
       <c r="F57" s="5" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="28.5">
+    <row r="58" spans="1:6" ht="27.6">
       <c r="A58" s="8">
         <v>14</v>
       </c>
@@ -2367,21 +2287,19 @@
         <v>28</v>
       </c>
       <c r="C58" s="8">
-        <f t="shared" si="4"/>
-        <v>14.499999999999998</v>
+        <v>14.5</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>181</v>
       </c>
       <c r="E58" s="8">
-        <f t="shared" si="1"/>
         <v>57</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="28.5">
+    <row r="59" spans="1:6" ht="27.6">
       <c r="A59" s="8">
         <v>14</v>
       </c>
@@ -2389,21 +2307,19 @@
         <v>28</v>
       </c>
       <c r="C59" s="8">
-        <f t="shared" si="4"/>
-        <v>14.599999999999998</v>
+        <v>14.6</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>182</v>
       </c>
       <c r="E59" s="8">
-        <f t="shared" si="1"/>
         <v>58</v>
       </c>
       <c r="F59" s="5" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="42.75">
+    <row r="60" spans="1:6" ht="41.4">
       <c r="A60" s="8">
         <v>14</v>
       </c>
@@ -2411,21 +2327,19 @@
         <v>28</v>
       </c>
       <c r="C60" s="8">
-        <f t="shared" si="4"/>
-        <v>14.699999999999998</v>
+        <v>14.7</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>183</v>
       </c>
       <c r="E60" s="8">
-        <f t="shared" si="1"/>
         <v>59</v>
       </c>
       <c r="F60" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="28.5">
+    <row r="61" spans="1:6" ht="27.6">
       <c r="A61" s="8">
         <v>14</v>
       </c>
@@ -2433,21 +2347,19 @@
         <v>28</v>
       </c>
       <c r="C61" s="8">
-        <f t="shared" si="4"/>
-        <v>14.799999999999997</v>
+        <v>14.8</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>184</v>
       </c>
       <c r="E61" s="8">
-        <f t="shared" si="1"/>
         <v>60</v>
       </c>
       <c r="F61" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="28.5">
+    <row r="62" spans="1:6" ht="27.6">
       <c r="A62" s="8">
         <v>14</v>
       </c>
@@ -2455,21 +2367,19 @@
         <v>28</v>
       </c>
       <c r="C62" s="8">
-        <f t="shared" si="4"/>
-        <v>14.899999999999997</v>
+        <v>14.9</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>192</v>
       </c>
       <c r="E62" s="8">
-        <f t="shared" si="1"/>
         <v>61</v>
       </c>
       <c r="F62" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="57">
+    <row r="63" spans="1:6" ht="55.2">
       <c r="A63" s="8">
         <v>14</v>
       </c>
@@ -2483,14 +2393,13 @@
         <v>185</v>
       </c>
       <c r="E63" s="8">
-        <f t="shared" si="1"/>
         <v>62</v>
       </c>
       <c r="F63" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="42.75">
+    <row r="64" spans="1:6" ht="41.4">
       <c r="A64" s="8">
         <v>14</v>
       </c>
@@ -2504,14 +2413,13 @@
         <v>186</v>
       </c>
       <c r="E64" s="8">
-        <f t="shared" si="1"/>
         <v>63</v>
       </c>
       <c r="F64" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="28.5">
+    <row r="65" spans="1:6" ht="27.6">
       <c r="A65" s="8">
         <v>14</v>
       </c>
@@ -2525,14 +2433,13 @@
         <v>187</v>
       </c>
       <c r="E65" s="8">
-        <f t="shared" si="1"/>
         <v>64</v>
       </c>
       <c r="F65" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="42.75">
+    <row r="66" spans="1:6" ht="41.4">
       <c r="A66" s="8">
         <v>14</v>
       </c>
@@ -2546,14 +2453,13 @@
         <v>188</v>
       </c>
       <c r="E66" s="8">
-        <f t="shared" si="1"/>
         <v>65</v>
       </c>
       <c r="F66" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="28.5">
+    <row r="67" spans="1:6" ht="27.6">
       <c r="A67" s="8">
         <v>14</v>
       </c>
@@ -2567,14 +2473,13 @@
         <v>189</v>
       </c>
       <c r="E67" s="8">
-        <f t="shared" si="1"/>
         <v>66</v>
       </c>
       <c r="F67" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="28.5">
+    <row r="68" spans="1:6" ht="27.6">
       <c r="A68" s="8">
         <v>14</v>
       </c>
@@ -2588,14 +2493,13 @@
         <v>190</v>
       </c>
       <c r="E68" s="8">
-        <f t="shared" ref="E68:E94" si="5">E67+1</f>
         <v>67</v>
       </c>
       <c r="F68" s="5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="28.5">
+    <row r="69" spans="1:6" ht="27.6">
       <c r="A69" s="8">
         <v>14</v>
       </c>
@@ -2609,14 +2513,13 @@
         <v>193</v>
       </c>
       <c r="E69" s="8">
-        <f t="shared" si="5"/>
         <v>68</v>
       </c>
       <c r="F69" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="42.75">
+    <row r="70" spans="1:6" ht="41.4">
       <c r="A70" s="8">
         <v>14</v>
       </c>
@@ -2630,14 +2533,13 @@
         <v>194</v>
       </c>
       <c r="E70" s="8">
-        <f t="shared" si="5"/>
         <v>69</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="42.75">
+    <row r="71" spans="1:6" ht="41.4">
       <c r="A71" s="8">
         <v>15</v>
       </c>
@@ -2651,14 +2553,13 @@
         <v>195</v>
       </c>
       <c r="E71" s="8">
-        <f t="shared" si="5"/>
         <v>70</v>
       </c>
       <c r="F71" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="28.5">
+    <row r="72" spans="1:6" ht="27.6">
       <c r="A72" s="8">
         <v>16</v>
       </c>
@@ -2672,7 +2573,6 @@
         <v>196</v>
       </c>
       <c r="E72" s="8">
-        <f t="shared" si="5"/>
         <v>71</v>
       </c>
       <c r="F72" s="4" t="s">
@@ -2687,14 +2587,12 @@
         <v>13</v>
       </c>
       <c r="C73" s="8">
-        <f>C72+0.1</f>
-        <v>16.200000000000003</v>
+        <v>16.2</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>197</v>
       </c>
       <c r="E73" s="8">
-        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="F73" s="4" t="s">
@@ -2709,21 +2607,19 @@
         <v>13</v>
       </c>
       <c r="C74" s="8">
-        <f t="shared" ref="C74:C80" si="6">C73+0.1</f>
-        <v>16.300000000000004</v>
+        <v>16.3</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>198</v>
       </c>
       <c r="E74" s="8">
-        <f t="shared" si="5"/>
         <v>73</v>
       </c>
       <c r="F74" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="28.5">
+    <row r="75" spans="1:6" ht="27.6">
       <c r="A75" s="8">
         <v>16</v>
       </c>
@@ -2731,14 +2627,12 @@
         <v>13</v>
       </c>
       <c r="C75" s="8">
-        <f t="shared" si="6"/>
-        <v>16.400000000000006</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>199</v>
       </c>
       <c r="E75" s="8">
-        <f t="shared" si="5"/>
         <v>74</v>
       </c>
       <c r="F75" s="5" t="s">
@@ -2753,21 +2647,19 @@
         <v>13</v>
       </c>
       <c r="C76" s="8">
-        <f t="shared" si="6"/>
-        <v>16.500000000000007</v>
+        <v>16.5</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>200</v>
       </c>
       <c r="E76" s="8">
-        <f t="shared" si="5"/>
         <v>75</v>
       </c>
       <c r="F76" s="4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="28.5">
+    <row r="77" spans="1:6" ht="27.6">
       <c r="A77" s="8">
         <v>16</v>
       </c>
@@ -2775,21 +2667,19 @@
         <v>13</v>
       </c>
       <c r="C77" s="8">
-        <f t="shared" si="6"/>
-        <v>16.600000000000009</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>201</v>
       </c>
       <c r="E77" s="8">
-        <f t="shared" si="5"/>
         <v>76</v>
       </c>
       <c r="F77" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="28.5">
+    <row r="78" spans="1:6" ht="27.6">
       <c r="A78" s="8">
         <v>16</v>
       </c>
@@ -2797,21 +2687,19 @@
         <v>13</v>
       </c>
       <c r="C78" s="8">
-        <f t="shared" si="6"/>
-        <v>16.70000000000001</v>
+        <v>16.7</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>202</v>
       </c>
       <c r="E78" s="8">
-        <f t="shared" si="5"/>
         <v>77</v>
       </c>
       <c r="F78" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="57">
+    <row r="79" spans="1:6" ht="55.2">
       <c r="A79" s="8">
         <v>16</v>
       </c>
@@ -2819,21 +2707,19 @@
         <v>13</v>
       </c>
       <c r="C79" s="8">
-        <f t="shared" si="6"/>
-        <v>16.800000000000011</v>
+        <v>16.8</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>203</v>
       </c>
       <c r="E79" s="8">
-        <f t="shared" si="5"/>
         <v>78</v>
       </c>
       <c r="F79" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="42.75">
+    <row r="80" spans="1:6" ht="41.4">
       <c r="A80" s="8">
         <v>16</v>
       </c>
@@ -2841,21 +2727,19 @@
         <v>13</v>
       </c>
       <c r="C80" s="8">
-        <f t="shared" si="6"/>
-        <v>16.900000000000013</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>204</v>
       </c>
       <c r="E80" s="8">
-        <f t="shared" si="5"/>
         <v>79</v>
       </c>
       <c r="F80" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="42.75">
+    <row r="81" spans="1:6" ht="41.4">
       <c r="A81" s="8">
         <v>16</v>
       </c>
@@ -2869,14 +2753,13 @@
         <v>205</v>
       </c>
       <c r="E81" s="8">
-        <f t="shared" si="5"/>
         <v>80</v>
       </c>
       <c r="F81" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="42.75">
+    <row r="82" spans="1:6" ht="41.4">
       <c r="A82" s="8">
         <v>16</v>
       </c>
@@ -2890,14 +2773,13 @@
         <v>206</v>
       </c>
       <c r="E82" s="8">
-        <f t="shared" si="5"/>
         <v>81</v>
       </c>
       <c r="F82" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="42.75">
+    <row r="83" spans="1:6" ht="27.6">
       <c r="A83" s="8">
         <v>17</v>
       </c>
@@ -2911,14 +2793,13 @@
         <v>207</v>
       </c>
       <c r="E83" s="8">
-        <f t="shared" si="5"/>
         <v>82</v>
       </c>
       <c r="F83" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="42.75">
+    <row r="84" spans="1:6" ht="27.6">
       <c r="A84" s="8">
         <v>17</v>
       </c>
@@ -2926,14 +2807,12 @@
         <v>84</v>
       </c>
       <c r="C84" s="8">
-        <f>C83+0.1</f>
-        <v>17.200000000000003</v>
+        <v>17.2</v>
       </c>
       <c r="D84" s="4" t="s">
         <v>208</v>
       </c>
       <c r="E84" s="8">
-        <f t="shared" si="5"/>
         <v>83</v>
       </c>
       <c r="F84" s="5" t="s">
@@ -2948,21 +2827,19 @@
         <v>84</v>
       </c>
       <c r="C85" s="8">
-        <f t="shared" ref="C85:C91" si="7">C84+0.1</f>
-        <v>17.300000000000004</v>
+        <v>17.3</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>210</v>
       </c>
       <c r="E85" s="8">
-        <f t="shared" si="5"/>
         <v>84</v>
       </c>
       <c r="F85" s="4" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="28.5">
+    <row r="86" spans="1:6" ht="27.6">
       <c r="A86" s="8">
         <v>17</v>
       </c>
@@ -2970,14 +2847,12 @@
         <v>84</v>
       </c>
       <c r="C86" s="8">
-        <f t="shared" si="7"/>
-        <v>17.400000000000006</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="D86" s="4" t="s">
         <v>211</v>
       </c>
       <c r="E86" s="8">
-        <f t="shared" si="5"/>
         <v>85</v>
       </c>
       <c r="F86" s="4" t="s">
@@ -2992,21 +2867,19 @@
         <v>84</v>
       </c>
       <c r="C87" s="8">
-        <f t="shared" si="7"/>
-        <v>17.500000000000007</v>
+        <v>17.5</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>213</v>
       </c>
       <c r="E87" s="8">
-        <f t="shared" si="5"/>
         <v>86</v>
       </c>
       <c r="F87" s="4" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="42.75">
+    <row r="88" spans="1:6" ht="41.4">
       <c r="A88" s="8">
         <v>17</v>
       </c>
@@ -3014,21 +2887,19 @@
         <v>84</v>
       </c>
       <c r="C88" s="8">
-        <f t="shared" si="7"/>
-        <v>17.600000000000009</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="D88" s="4" t="s">
         <v>214</v>
       </c>
       <c r="E88" s="8">
-        <f t="shared" si="5"/>
         <v>87</v>
       </c>
       <c r="F88" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="1:6" ht="28.5">
+    <row r="89" spans="1:6" ht="27.6">
       <c r="A89" s="8">
         <v>17</v>
       </c>
@@ -3036,21 +2907,19 @@
         <v>84</v>
       </c>
       <c r="C89" s="8">
-        <f t="shared" si="7"/>
-        <v>17.70000000000001</v>
+        <v>17.7</v>
       </c>
       <c r="D89" s="4" t="s">
         <v>215</v>
       </c>
       <c r="E89" s="8">
-        <f t="shared" si="5"/>
         <v>88</v>
       </c>
       <c r="F89" s="4" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="28.5">
+    <row r="90" spans="1:6" ht="27.6">
       <c r="A90" s="8">
         <v>17</v>
       </c>
@@ -3058,21 +2927,19 @@
         <v>84</v>
       </c>
       <c r="C90" s="8">
-        <f t="shared" si="7"/>
-        <v>17.800000000000011</v>
+        <v>17.8</v>
       </c>
       <c r="D90" s="4" t="s">
         <v>217</v>
       </c>
       <c r="E90" s="8">
-        <f t="shared" si="5"/>
         <v>89</v>
       </c>
       <c r="F90" s="4" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="91" spans="1:6" ht="42.75">
+    <row r="91" spans="1:6" ht="41.4">
       <c r="A91" s="8">
         <v>17</v>
       </c>
@@ -3080,14 +2947,12 @@
         <v>84</v>
       </c>
       <c r="C91" s="8">
-        <f t="shared" si="7"/>
-        <v>17.900000000000013</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>218</v>
       </c>
       <c r="E91" s="8">
-        <f t="shared" si="5"/>
         <v>90</v>
       </c>
       <c r="F91" s="4" t="s">
@@ -3108,14 +2973,13 @@
         <v>219</v>
       </c>
       <c r="E92" s="8">
-        <f t="shared" si="5"/>
         <v>91</v>
       </c>
       <c r="F92" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="28.5">
+    <row r="93" spans="1:6" ht="27.6">
       <c r="A93" s="8">
         <v>18</v>
       </c>
@@ -3123,14 +2987,12 @@
         <v>86</v>
       </c>
       <c r="C93" s="8">
-        <f t="shared" ref="A71:C94" si="8">C92+1</f>
         <v>18.100000000000001</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>220</v>
       </c>
       <c r="E93" s="8">
-        <f t="shared" si="5"/>
         <v>92</v>
       </c>
       <c r="F93" s="4" t="s">
@@ -3145,14 +3007,12 @@
         <v>94</v>
       </c>
       <c r="C94" s="8">
-        <f t="shared" si="8"/>
         <v>19.100000000000001</v>
       </c>
       <c r="D94" s="4" t="s">
         <v>221</v>
       </c>
       <c r="E94" s="8">
-        <f t="shared" si="5"/>
         <v>93</v>
       </c>
       <c r="F94" s="5" t="s">

</xml_diff>

<commit_message>
added unfirm cide for complaicn eof pci , cobit and soc2
</commit_message>
<xml_diff>
--- a/Audit_Code/public/SOC2_Type2.xlsx
+++ b/Audit_Code/public/SOC2_Type2.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muhammad.abdullah\Documents\Compliance\Audit_Code\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\97154\Downloads\KAB\standardssheetstobefixed\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B0BDE90-600F-48EC-BC24-AE22D054F387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15348" windowHeight="4632"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,17 +23,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -361,9 +351,6 @@
     <t>IT Operational Anomalies Reporting</t>
   </si>
   <si>
-    <t>Trust Criteria Domain</t>
-  </si>
-  <si>
     <t>Trust Criteria Principle</t>
   </si>
   <si>
@@ -704,13 +691,16 @@
   </si>
   <si>
     <t>Regular vulnerability scans.</t>
+  </si>
+  <si>
+    <t>Domain</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1132,34 +1122,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F94"/>
-  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.09765625" style="9"/>
-    <col min="2" max="2" width="29.59765625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="8.8984375" style="9" customWidth="1"/>
-    <col min="4" max="4" width="37.09765625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="7.8984375" style="9" customWidth="1"/>
-    <col min="6" max="6" width="107.09765625" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.09765625" style="2"/>
+    <col min="1" max="1" width="9.140625" style="9"/>
+    <col min="2" max="2" width="29.5703125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="9" customWidth="1"/>
+    <col min="4" max="4" width="37.140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="7.85546875" style="9" customWidth="1"/>
+    <col min="6" max="6" width="107.140625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1">
+    <row r="1" spans="1:6" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="7"/>
       <c r="B1" s="3" t="s">
-        <v>107</v>
+        <v>221</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -1170,7 +1160,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E2" s="8">
         <v>1</v>
@@ -1179,7 +1169,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -1190,7 +1180,7 @@
         <v>1.2</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E3" s="8">
         <v>2</v>
@@ -1199,7 +1189,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="27.6">
+    <row r="4" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>2</v>
       </c>
@@ -1210,7 +1200,7 @@
         <v>2.1</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E4" s="8">
         <v>3</v>
@@ -1219,7 +1209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
         <v>2</v>
       </c>
@@ -1230,7 +1220,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E5" s="8">
         <v>4</v>
@@ -1239,7 +1229,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="8">
         <v>2</v>
       </c>
@@ -1250,7 +1240,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E6" s="8">
         <v>5</v>
@@ -1259,7 +1249,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
         <v>2</v>
       </c>
@@ -1270,7 +1260,7 @@
         <v>2.4</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E7" s="8">
         <v>6</v>
@@ -1279,7 +1269,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="27.6">
+    <row r="8" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
         <v>2</v>
       </c>
@@ -1290,7 +1280,7 @@
         <v>2.5</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E8" s="8">
         <v>7</v>
@@ -1299,7 +1289,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>2</v>
       </c>
@@ -1310,7 +1300,7 @@
         <v>2.6</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E9" s="8">
         <v>8</v>
@@ -1319,7 +1309,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="41.4">
+    <row r="10" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
         <v>2</v>
       </c>
@@ -1330,7 +1320,7 @@
         <v>2.7</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E10" s="8">
         <v>9</v>
@@ -1339,7 +1329,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="27.6">
+    <row r="11" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>2</v>
       </c>
@@ -1350,7 +1340,7 @@
         <v>2.8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E11" s="8">
         <v>10</v>
@@ -1359,7 +1349,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="41.4">
+    <row r="12" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
         <v>3</v>
       </c>
@@ -1370,7 +1360,7 @@
         <v>3.1</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E12" s="8">
         <v>11</v>
@@ -1379,7 +1369,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="27.6">
+    <row r="13" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
         <v>3</v>
       </c>
@@ -1390,7 +1380,7 @@
         <v>3.2</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E13" s="8">
         <v>12</v>
@@ -1399,7 +1389,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
         <v>3</v>
       </c>
@@ -1410,7 +1400,7 @@
         <v>3.3</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E14" s="8">
         <v>13</v>
@@ -1419,7 +1409,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
         <v>3</v>
       </c>
@@ -1430,7 +1420,7 @@
         <v>3.4</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E15" s="8">
         <v>14</v>
@@ -1439,7 +1429,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="27.6">
+    <row r="16" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
         <v>3</v>
       </c>
@@ -1450,7 +1440,7 @@
         <v>3.5</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E16" s="8">
         <v>15</v>
@@ -1459,7 +1449,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="41.4">
+    <row r="17" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
         <v>3</v>
       </c>
@@ -1470,7 +1460,7 @@
         <v>3.6</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E17" s="8">
         <v>16</v>
@@ -1479,7 +1469,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
         <v>4</v>
       </c>
@@ -1490,7 +1480,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E18" s="8">
         <v>17</v>
@@ -1499,7 +1489,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="27.6">
+    <row r="19" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
         <v>4</v>
       </c>
@@ -1510,7 +1500,7 @@
         <v>4.2</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E19" s="8">
         <v>18</v>
@@ -1519,7 +1509,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="27.6">
+    <row r="20" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
         <v>4</v>
       </c>
@@ -1530,7 +1520,7 @@
         <v>4.3</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E20" s="8">
         <v>19</v>
@@ -1539,7 +1529,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="41.4">
+    <row r="21" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
         <v>4</v>
       </c>
@@ -1550,7 +1540,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E21" s="8">
         <v>20</v>
@@ -1559,7 +1549,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="27.6">
+    <row r="22" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
         <v>4</v>
       </c>
@@ -1570,7 +1560,7 @@
         <v>4.5</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E22" s="8">
         <v>21</v>
@@ -1579,7 +1569,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="27.6">
+    <row r="23" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
         <v>4</v>
       </c>
@@ -1590,16 +1580,16 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E23" s="8">
         <v>22</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="41.4">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
         <v>4</v>
       </c>
@@ -1610,16 +1600,16 @@
         <v>4.7</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E24" s="8">
         <v>23</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="27.6">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
         <v>4</v>
       </c>
@@ -1630,7 +1620,7 @@
         <v>4.8</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E25" s="8">
         <v>24</v>
@@ -1639,7 +1629,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="27.6">
+    <row r="26" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
         <v>5</v>
       </c>
@@ -1650,7 +1640,7 @@
         <v>5</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E26" s="8">
         <v>25</v>
@@ -1659,7 +1649,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="27.6">
+    <row r="27" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
         <v>5</v>
       </c>
@@ -1670,7 +1660,7 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E27" s="8">
         <v>26</v>
@@ -1679,7 +1669,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="41.4">
+    <row r="28" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
         <v>5</v>
       </c>
@@ -1690,7 +1680,7 @@
         <v>5.2</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E28" s="8">
         <v>27</v>
@@ -1699,7 +1689,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="27.6">
+    <row r="29" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
         <v>5</v>
       </c>
@@ -1710,7 +1700,7 @@
         <v>5.3</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E29" s="8">
         <v>28</v>
@@ -1719,7 +1709,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="27.6">
+    <row r="30" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
         <v>5</v>
       </c>
@@ -1730,7 +1720,7 @@
         <v>5.4</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E30" s="8">
         <v>29</v>
@@ -1739,7 +1729,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
         <v>5</v>
       </c>
@@ -1750,7 +1740,7 @@
         <v>5.5</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E31" s="8">
         <v>30</v>
@@ -1759,7 +1749,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="27.6">
+    <row r="32" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
         <v>5</v>
       </c>
@@ -1770,7 +1760,7 @@
         <v>5.6</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E32" s="8">
         <v>31</v>
@@ -1779,7 +1769,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
         <v>5</v>
       </c>
@@ -1790,7 +1780,7 @@
         <v>5.7</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E33" s="8">
         <v>32</v>
@@ -1799,7 +1789,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="27.6">
+    <row r="34" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A34" s="8">
         <v>5</v>
       </c>
@@ -1810,7 +1800,7 @@
         <v>5.8</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E34" s="8">
         <v>33</v>
@@ -1819,7 +1809,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
         <v>5</v>
       </c>
@@ -1830,7 +1820,7 @@
         <v>5.9</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E35" s="8">
         <v>34</v>
@@ -1839,7 +1829,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="8">
         <v>6</v>
       </c>
@@ -1850,7 +1840,7 @@
         <v>6.1</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E36" s="8">
         <v>35</v>
@@ -1859,7 +1849,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
         <v>7</v>
       </c>
@@ -1870,7 +1860,7 @@
         <v>7.1</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E37" s="8">
         <v>36</v>
@@ -1879,7 +1869,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="27.6">
+    <row r="38" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
         <v>8</v>
       </c>
@@ -1890,7 +1880,7 @@
         <v>8.1</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E38" s="8">
         <v>37</v>
@@ -1899,7 +1889,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="27.6">
+    <row r="39" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
         <v>8</v>
       </c>
@@ -1910,7 +1900,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E39" s="8">
         <v>38</v>
@@ -1919,7 +1909,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="27.6">
+    <row r="40" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
         <v>8</v>
       </c>
@@ -1930,7 +1920,7 @@
         <v>8.3000000000000007</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E40" s="8">
         <v>39</v>
@@ -1939,7 +1929,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="27.6">
+    <row r="41" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A41" s="8">
         <v>8</v>
       </c>
@@ -1950,7 +1940,7 @@
         <v>8.4</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E41" s="8">
         <v>40</v>
@@ -1959,7 +1949,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="27.6">
+    <row r="42" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
         <v>8</v>
       </c>
@@ -1970,7 +1960,7 @@
         <v>8.5</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E42" s="8">
         <v>41</v>
@@ -1979,7 +1969,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="27.6">
+    <row r="43" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A43" s="8">
         <v>8</v>
       </c>
@@ -1990,7 +1980,7 @@
         <v>8.6</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E43" s="8">
         <v>42</v>
@@ -1999,7 +1989,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="27.6">
+    <row r="44" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A44" s="8">
         <v>8</v>
       </c>
@@ -2010,7 +2000,7 @@
         <v>8.6999999999999993</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E44" s="8">
         <v>43</v>
@@ -2019,7 +2009,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="27.6">
+    <row r="45" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A45" s="8">
         <v>8</v>
       </c>
@@ -2030,7 +2020,7 @@
         <v>8.8000000000000007</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E45" s="8">
         <v>44</v>
@@ -2039,7 +2029,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="27.6">
+    <row r="46" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
         <v>8</v>
       </c>
@@ -2050,7 +2040,7 @@
         <v>8.9</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E46" s="8">
         <v>45</v>
@@ -2059,7 +2049,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="27.6">
+    <row r="47" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
         <v>8</v>
       </c>
@@ -2067,10 +2057,10 @@
         <v>90</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E47" s="8">
         <v>46</v>
@@ -2079,7 +2069,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="27.6">
+    <row r="48" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A48" s="8">
         <v>8</v>
       </c>
@@ -2087,10 +2077,10 @@
         <v>90</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E48" s="8">
         <v>47</v>
@@ -2099,7 +2089,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="27.6">
+    <row r="49" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
         <v>9</v>
       </c>
@@ -2110,16 +2100,16 @@
         <v>9.1</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E49" s="8">
         <v>48</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="27.6">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
         <v>10</v>
       </c>
@@ -2130,7 +2120,7 @@
         <v>10.1</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E50" s="8">
         <v>49</v>
@@ -2139,7 +2129,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="27.6">
+    <row r="51" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A51" s="8">
         <v>11</v>
       </c>
@@ -2150,7 +2140,7 @@
         <v>11.1</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E51" s="8">
         <v>50</v>
@@ -2159,7 +2149,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="27.6">
+    <row r="52" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
         <v>12</v>
       </c>
@@ -2170,7 +2160,7 @@
         <v>12.1</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E52" s="8">
         <v>51</v>
@@ -2179,7 +2169,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="41.4">
+    <row r="53" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A53" s="8">
         <v>13</v>
       </c>
@@ -2190,7 +2180,7 @@
         <v>13.1</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E53" s="8">
         <v>52</v>
@@ -2199,7 +2189,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="41.4">
+    <row r="54" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
         <v>14</v>
       </c>
@@ -2210,7 +2200,7 @@
         <v>14.1</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E54" s="8">
         <v>53</v>
@@ -2219,7 +2209,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="27.6">
+    <row r="55" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
         <v>14</v>
       </c>
@@ -2230,7 +2220,7 @@
         <v>14.2</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E55" s="8">
         <v>54</v>
@@ -2239,7 +2229,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="27.6">
+    <row r="56" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A56" s="8">
         <v>14</v>
       </c>
@@ -2250,7 +2240,7 @@
         <v>14.3</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E56" s="8">
         <v>55</v>
@@ -2259,7 +2249,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="27.6">
+    <row r="57" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
         <v>14</v>
       </c>
@@ -2270,7 +2260,7 @@
         <v>14.4</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E57" s="8">
         <v>56</v>
@@ -2279,7 +2269,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="27.6">
+    <row r="58" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A58" s="8">
         <v>14</v>
       </c>
@@ -2290,7 +2280,7 @@
         <v>14.5</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E58" s="8">
         <v>57</v>
@@ -2299,7 +2289,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="27.6">
+    <row r="59" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A59" s="8">
         <v>14</v>
       </c>
@@ -2310,7 +2300,7 @@
         <v>14.6</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E59" s="8">
         <v>58</v>
@@ -2319,7 +2309,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="41.4">
+    <row r="60" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A60" s="8">
         <v>14</v>
       </c>
@@ -2330,7 +2320,7 @@
         <v>14.7</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E60" s="8">
         <v>59</v>
@@ -2339,7 +2329,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="27.6">
+    <row r="61" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A61" s="8">
         <v>14</v>
       </c>
@@ -2350,7 +2340,7 @@
         <v>14.8</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E61" s="8">
         <v>60</v>
@@ -2359,7 +2349,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="27.6">
+    <row r="62" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A62" s="8">
         <v>14</v>
       </c>
@@ -2370,7 +2360,7 @@
         <v>14.9</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E62" s="8">
         <v>61</v>
@@ -2379,7 +2369,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="55.2">
+    <row r="63" spans="1:6" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A63" s="8">
         <v>14</v>
       </c>
@@ -2387,10 +2377,10 @@
         <v>28</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E63" s="8">
         <v>62</v>
@@ -2399,7 +2389,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="41.4">
+    <row r="64" spans="1:6" ht="57" x14ac:dyDescent="0.25">
       <c r="A64" s="8">
         <v>14</v>
       </c>
@@ -2407,10 +2397,10 @@
         <v>28</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E64" s="8">
         <v>63</v>
@@ -2419,7 +2409,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="27.6">
+    <row r="65" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A65" s="8">
         <v>14</v>
       </c>
@@ -2427,10 +2417,10 @@
         <v>28</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E65" s="8">
         <v>64</v>
@@ -2439,7 +2429,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="41.4">
+    <row r="66" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A66" s="8">
         <v>14</v>
       </c>
@@ -2447,10 +2437,10 @@
         <v>28</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E66" s="8">
         <v>65</v>
@@ -2459,7 +2449,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="27.6">
+    <row r="67" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
         <v>14</v>
       </c>
@@ -2467,10 +2457,10 @@
         <v>28</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E67" s="8">
         <v>66</v>
@@ -2479,7 +2469,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="27.6">
+    <row r="68" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
         <v>14</v>
       </c>
@@ -2487,10 +2477,10 @@
         <v>28</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E68" s="8">
         <v>67</v>
@@ -2499,7 +2489,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="27.6">
+    <row r="69" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A69" s="8">
         <v>14</v>
       </c>
@@ -2507,19 +2497,19 @@
         <v>28</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E69" s="8">
         <v>68</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="41.4">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A70" s="8">
         <v>14</v>
       </c>
@@ -2527,10 +2517,10 @@
         <v>28</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E70" s="8">
         <v>69</v>
@@ -2539,7 +2529,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="41.4">
+    <row r="71" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A71" s="8">
         <v>15</v>
       </c>
@@ -2550,7 +2540,7 @@
         <v>15.1</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E71" s="8">
         <v>70</v>
@@ -2559,7 +2549,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="27.6">
+    <row r="72" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A72" s="8">
         <v>16</v>
       </c>
@@ -2570,7 +2560,7 @@
         <v>16.100000000000001</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E72" s="8">
         <v>71</v>
@@ -2579,7 +2569,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="8">
         <v>16</v>
       </c>
@@ -2590,7 +2580,7 @@
         <v>16.2</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E73" s="8">
         <v>72</v>
@@ -2599,7 +2589,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A74" s="8">
         <v>16</v>
       </c>
@@ -2610,7 +2600,7 @@
         <v>16.3</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E74" s="8">
         <v>73</v>
@@ -2619,7 +2609,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="27.6">
+    <row r="75" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A75" s="8">
         <v>16</v>
       </c>
@@ -2630,7 +2620,7 @@
         <v>16.399999999999999</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E75" s="8">
         <v>74</v>
@@ -2639,7 +2629,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A76" s="8">
         <v>16</v>
       </c>
@@ -2650,7 +2640,7 @@
         <v>16.5</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E76" s="8">
         <v>75</v>
@@ -2659,7 +2649,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="27.6">
+    <row r="77" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A77" s="8">
         <v>16</v>
       </c>
@@ -2670,7 +2660,7 @@
         <v>16.600000000000001</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E77" s="8">
         <v>76</v>
@@ -2679,7 +2669,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="27.6">
+    <row r="78" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A78" s="8">
         <v>16</v>
       </c>
@@ -2690,7 +2680,7 @@
         <v>16.7</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E78" s="8">
         <v>77</v>
@@ -2699,7 +2689,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="55.2">
+    <row r="79" spans="1:6" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A79" s="8">
         <v>16</v>
       </c>
@@ -2710,7 +2700,7 @@
         <v>16.8</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E79" s="8">
         <v>78</v>
@@ -2719,7 +2709,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="41.4">
+    <row r="80" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A80" s="8">
         <v>16</v>
       </c>
@@ -2730,7 +2720,7 @@
         <v>16.899999999999999</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E80" s="8">
         <v>79</v>
@@ -2739,7 +2729,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="41.4">
+    <row r="81" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A81" s="8">
         <v>16</v>
       </c>
@@ -2747,10 +2737,10 @@
         <v>13</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E81" s="8">
         <v>80</v>
@@ -2759,7 +2749,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="41.4">
+    <row r="82" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A82" s="8">
         <v>16</v>
       </c>
@@ -2767,10 +2757,10 @@
         <v>13</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E82" s="8">
         <v>81</v>
@@ -2779,7 +2769,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="27.6">
+    <row r="83" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A83" s="8">
         <v>17</v>
       </c>
@@ -2790,7 +2780,7 @@
         <v>17.100000000000001</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E83" s="8">
         <v>82</v>
@@ -2799,7 +2789,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="27.6">
+    <row r="84" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A84" s="8">
         <v>17</v>
       </c>
@@ -2810,7 +2800,7 @@
         <v>17.2</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E84" s="8">
         <v>83</v>
@@ -2819,7 +2809,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="8">
         <v>17</v>
       </c>
@@ -2830,16 +2820,16 @@
         <v>17.3</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E85" s="8">
         <v>84</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" ht="27.6">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A86" s="8">
         <v>17</v>
       </c>
@@ -2850,7 +2840,7 @@
         <v>17.399999999999999</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E86" s="8">
         <v>85</v>
@@ -2859,7 +2849,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="8">
         <v>17</v>
       </c>
@@ -2870,16 +2860,16 @@
         <v>17.5</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E87" s="8">
         <v>86</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" ht="41.4">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A88" s="8">
         <v>17</v>
       </c>
@@ -2890,7 +2880,7 @@
         <v>17.600000000000001</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E88" s="8">
         <v>87</v>
@@ -2899,7 +2889,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="1:6" ht="27.6">
+    <row r="89" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A89" s="8">
         <v>17</v>
       </c>
@@ -2910,7 +2900,7 @@
         <v>17.7</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E89" s="8">
         <v>88</v>
@@ -2919,7 +2909,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="27.6">
+    <row r="90" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A90" s="8">
         <v>17</v>
       </c>
@@ -2930,16 +2920,16 @@
         <v>17.8</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E90" s="8">
         <v>89</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" ht="41.4">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="57" x14ac:dyDescent="0.25">
       <c r="A91" s="8">
         <v>17</v>
       </c>
@@ -2950,7 +2940,7 @@
         <v>17.899999999999999</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E91" s="8">
         <v>90</v>
@@ -2959,7 +2949,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A92" s="8">
         <v>17</v>
       </c>
@@ -2967,10 +2957,10 @@
         <v>84</v>
       </c>
       <c r="C92" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E92" s="8">
         <v>91</v>
@@ -2979,7 +2969,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="27.6">
+    <row r="93" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A93" s="8">
         <v>18</v>
       </c>
@@ -2990,7 +2980,7 @@
         <v>18.100000000000001</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E93" s="8">
         <v>92</v>
@@ -2999,7 +2989,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="8">
         <v>19</v>
       </c>
@@ -3010,7 +3000,7 @@
         <v>19.100000000000001</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E94" s="8">
         <v>93</v>
@@ -3020,8 +3010,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="D1:F94"/>
-  <sortState ref="C2:F113">
+  <autoFilter ref="D1:F94" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C2:F113">
     <sortCondition ref="D2:D113"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>